<commit_message>
updated r files and excel
</commit_message>
<xml_diff>
--- a/sub_pro_12_fifa_tm_analysis/datasets/caf_squad_value_mar_2026.xlsx
+++ b/sub_pro_12_fifa_tm_analysis/datasets/caf_squad_value_mar_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willy\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Files\sports_data_sci\sub_pro_12_fifa_tm_analysis\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44191EBA-BB4C-495F-A636-AE2859ACEC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479B9F56-89F7-4812-99EA-413D7A995C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{3AE42594-FA6B-4E9F-A1B4-60DE16C6AD15}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="309">
   <si>
     <t>Ranking</t>
   </si>
@@ -708,9 +708,6 @@
     <t>Value of Player</t>
   </si>
   <si>
-    <t>MVP:Total Squad Value Ratio</t>
-  </si>
-  <si>
     <t>Iliman Ndiaye</t>
   </si>
   <si>
@@ -943,6 +940,18 @@
   </si>
   <si>
     <t>€125k</t>
+  </si>
+  <si>
+    <t>€12.90m</t>
+  </si>
+  <si>
+    <t>Patson Daka</t>
+  </si>
+  <si>
+    <t>€12.00m</t>
+  </si>
+  <si>
+    <t>€561k</t>
   </si>
 </sst>
 </file>
@@ -1350,9 +1359,7 @@
       <c r="J1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>227</v>
-      </c>
+      <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -1380,10 +1387,10 @@
         <v>122</v>
       </c>
       <c r="I2" t="s">
+        <v>229</v>
+      </c>
+      <c r="J2" t="s">
         <v>230</v>
-      </c>
-      <c r="J2" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -1412,10 +1419,10 @@
         <v>118</v>
       </c>
       <c r="I3" t="s">
+        <v>227</v>
+      </c>
+      <c r="J3" t="s">
         <v>228</v>
-      </c>
-      <c r="J3" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
@@ -1444,10 +1451,10 @@
         <v>124</v>
       </c>
       <c r="I4" t="s">
+        <v>233</v>
+      </c>
+      <c r="J4" t="s">
         <v>234</v>
-      </c>
-      <c r="J4" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
@@ -1476,10 +1483,10 @@
         <v>126</v>
       </c>
       <c r="I5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -1508,10 +1515,10 @@
         <v>138</v>
       </c>
       <c r="I6" t="s">
+        <v>236</v>
+      </c>
+      <c r="J6" t="s">
         <v>237</v>
-      </c>
-      <c r="J6" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
@@ -1540,10 +1547,10 @@
         <v>120</v>
       </c>
       <c r="I7" t="s">
+        <v>231</v>
+      </c>
+      <c r="J7" t="s">
         <v>232</v>
-      </c>
-      <c r="J7" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -1572,10 +1579,10 @@
         <v>130</v>
       </c>
       <c r="I8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="J8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
@@ -1604,10 +1611,10 @@
         <v>146</v>
       </c>
       <c r="I9" t="s">
+        <v>239</v>
+      </c>
+      <c r="J9" t="s">
         <v>240</v>
-      </c>
-      <c r="J9" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
@@ -1636,10 +1643,10 @@
         <v>132</v>
       </c>
       <c r="I10" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
@@ -1668,10 +1675,10 @@
         <v>134</v>
       </c>
       <c r="I11" t="s">
+        <v>244</v>
+      </c>
+      <c r="J11" t="s">
         <v>245</v>
-      </c>
-      <c r="J11" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -1700,7 +1707,7 @@
         <v>152</v>
       </c>
       <c r="I12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J12" t="s">
         <v>124</v>
@@ -1732,10 +1739,10 @@
         <v>136</v>
       </c>
       <c r="I13" t="s">
+        <v>246</v>
+      </c>
+      <c r="J13" t="s">
         <v>247</v>
-      </c>
-      <c r="J13" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
@@ -1764,10 +1771,10 @@
         <v>148</v>
       </c>
       <c r="I14" t="s">
+        <v>252</v>
+      </c>
+      <c r="J14" t="s">
         <v>253</v>
-      </c>
-      <c r="J14" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
@@ -1796,10 +1803,10 @@
         <v>128</v>
       </c>
       <c r="I15" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J15" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
@@ -1828,10 +1835,10 @@
         <v>140</v>
       </c>
       <c r="I16" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J16" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -1860,10 +1867,10 @@
         <v>154</v>
       </c>
       <c r="I17" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="J17" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -1892,7 +1899,7 @@
         <v>183</v>
       </c>
       <c r="I18" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J18" t="s">
         <v>218</v>
@@ -1924,10 +1931,10 @@
         <v>144</v>
       </c>
       <c r="I19" t="s">
+        <v>249</v>
+      </c>
+      <c r="J19" t="s">
         <v>250</v>
-      </c>
-      <c r="J19" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -1943,23 +1950,23 @@
       <c r="D20" t="s">
         <v>31</v>
       </c>
-      <c r="E20" t="s">
-        <v>224</v>
-      </c>
-      <c r="F20" t="s">
-        <v>224</v>
+      <c r="E20">
+        <v>23</v>
+      </c>
+      <c r="F20">
+        <v>26.1</v>
       </c>
       <c r="G20" t="s">
-        <v>224</v>
+        <v>305</v>
       </c>
       <c r="H20" t="s">
-        <v>224</v>
+        <v>308</v>
       </c>
       <c r="I20" t="s">
-        <v>224</v>
+        <v>306</v>
       </c>
       <c r="J20" t="s">
-        <v>224</v>
+        <v>307</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -1988,7 +1995,7 @@
         <v>161</v>
       </c>
       <c r="I21" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="J21" t="s">
         <v>134</v>
@@ -2020,10 +2027,10 @@
         <v>154</v>
       </c>
       <c r="I22" t="s">
+        <v>260</v>
+      </c>
+      <c r="J22" t="s">
         <v>261</v>
-      </c>
-      <c r="J22" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -2052,7 +2059,7 @@
         <v>185</v>
       </c>
       <c r="I23" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J23" t="s">
         <v>206</v>
@@ -2084,10 +2091,10 @@
         <v>165</v>
       </c>
       <c r="I24" t="s">
+        <v>265</v>
+      </c>
+      <c r="J24" t="s">
         <v>266</v>
-      </c>
-      <c r="J24" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -2116,10 +2123,10 @@
         <v>175</v>
       </c>
       <c r="I25" t="s">
+        <v>270</v>
+      </c>
+      <c r="J25" t="s">
         <v>271</v>
-      </c>
-      <c r="J25" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
@@ -2148,10 +2155,10 @@
         <v>189</v>
       </c>
       <c r="I26" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J26" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -2180,10 +2187,10 @@
         <v>181</v>
       </c>
       <c r="I27" t="s">
+        <v>274</v>
+      </c>
+      <c r="J27" t="s">
         <v>275</v>
-      </c>
-      <c r="J27" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
@@ -2212,7 +2219,7 @@
         <v>177</v>
       </c>
       <c r="I28" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J28" t="s">
         <v>190</v>
@@ -2244,10 +2251,10 @@
         <v>173</v>
       </c>
       <c r="I29" t="s">
+        <v>268</v>
+      </c>
+      <c r="J29" t="s">
         <v>269</v>
-      </c>
-      <c r="J29" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
@@ -2276,7 +2283,7 @@
         <v>159</v>
       </c>
       <c r="I30" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J30" t="s">
         <v>190</v>
@@ -2308,10 +2315,10 @@
         <v>142</v>
       </c>
       <c r="I31" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="J31" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
@@ -2340,10 +2347,10 @@
         <v>199</v>
       </c>
       <c r="I32" t="s">
+        <v>287</v>
+      </c>
+      <c r="J32" t="s">
         <v>288</v>
-      </c>
-      <c r="J32" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
@@ -2372,10 +2379,10 @@
         <v>197</v>
       </c>
       <c r="I33" t="s">
+        <v>285</v>
+      </c>
+      <c r="J33" t="s">
         <v>286</v>
-      </c>
-      <c r="J33" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
@@ -2404,7 +2411,7 @@
         <v>179</v>
       </c>
       <c r="I34" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J34" t="s">
         <v>190</v>
@@ -2436,10 +2443,10 @@
         <v>157</v>
       </c>
       <c r="I35" t="s">
+        <v>258</v>
+      </c>
+      <c r="J35" t="s">
         <v>259</v>
-      </c>
-      <c r="J35" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
@@ -2468,10 +2475,10 @@
         <v>207</v>
       </c>
       <c r="I36" t="s">
+        <v>295</v>
+      </c>
+      <c r="J36" t="s">
         <v>296</v>
-      </c>
-      <c r="J36" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
@@ -2500,10 +2507,10 @@
         <v>193</v>
       </c>
       <c r="I37" t="s">
+        <v>281</v>
+      </c>
+      <c r="J37" t="s">
         <v>282</v>
-      </c>
-      <c r="J37" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
@@ -2532,7 +2539,7 @@
         <v>187</v>
       </c>
       <c r="I38" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J38" t="s">
         <v>206</v>
@@ -2564,10 +2571,10 @@
         <v>150</v>
       </c>
       <c r="I39" t="s">
+        <v>254</v>
+      </c>
+      <c r="J39" t="s">
         <v>255</v>
-      </c>
-      <c r="J39" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
@@ -2596,10 +2603,10 @@
         <v>205</v>
       </c>
       <c r="I40" t="s">
+        <v>293</v>
+      </c>
+      <c r="J40" t="s">
         <v>294</v>
-      </c>
-      <c r="J40" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
@@ -2628,10 +2635,10 @@
         <v>191</v>
       </c>
       <c r="I41" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J41" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
@@ -2660,7 +2667,7 @@
         <v>163</v>
       </c>
       <c r="I42" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="J42" t="s">
         <v>190</v>
@@ -2724,10 +2731,10 @@
         <v>201</v>
       </c>
       <c r="I44" t="s">
+        <v>289</v>
+      </c>
+      <c r="J44" t="s">
         <v>290</v>
-      </c>
-      <c r="J44" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
@@ -2756,10 +2763,10 @@
         <v>171</v>
       </c>
       <c r="I45" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J45" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
@@ -2788,10 +2795,10 @@
         <v>203</v>
       </c>
       <c r="I46" t="s">
+        <v>291</v>
+      </c>
+      <c r="J46" t="s">
         <v>292</v>
-      </c>
-      <c r="J46" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
@@ -2820,10 +2827,10 @@
         <v>215</v>
       </c>
       <c r="I47" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J47" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
@@ -2852,10 +2859,10 @@
         <v>211</v>
       </c>
       <c r="I48" t="s">
+        <v>298</v>
+      </c>
+      <c r="J48" t="s">
         <v>299</v>
-      </c>
-      <c r="J48" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
@@ -2916,10 +2923,10 @@
         <v>195</v>
       </c>
       <c r="I50" t="s">
+        <v>283</v>
+      </c>
+      <c r="J50" t="s">
         <v>284</v>
-      </c>
-      <c r="J50" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
@@ -2948,10 +2955,10 @@
         <v>213</v>
       </c>
       <c r="I51" t="s">
+        <v>300</v>
+      </c>
+      <c r="J51" t="s">
         <v>301</v>
-      </c>
-      <c r="J51" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
@@ -3012,10 +3019,10 @@
         <v>209</v>
       </c>
       <c r="I53" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J53" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
@@ -3044,13 +3051,14 @@
         <v>217</v>
       </c>
       <c r="I54" t="s">
+        <v>303</v>
+      </c>
+      <c r="J54" t="s">
         <v>304</v>
-      </c>
-      <c r="J54" t="s">
-        <v>305</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
squad value analysis and datasets
</commit_message>
<xml_diff>
--- a/sub_pro_12_fifa_tm_analysis/datasets/caf_squad_value_mar_2026.xlsx
+++ b/sub_pro_12_fifa_tm_analysis/datasets/caf_squad_value_mar_2026.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Files\sports_data_sci\sub_pro_12_fifa_tm_analysis\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479B9F56-89F7-4812-99EA-413D7A995C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F98FC1C3-22CD-46CB-8E50-911516F2DB45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{3AE42594-FA6B-4E9F-A1B4-60DE16C6AD15}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="536" xr2:uid="{3AE42594-FA6B-4E9F-A1B4-60DE16C6AD15}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$D$1:$D$54</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="310">
   <si>
     <t>Ranking</t>
   </si>
@@ -952,13 +955,16 @@
   </si>
   <si>
     <t>€561k</t>
+  </si>
+  <si>
+    <t>Players playing abroad (%)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -973,6 +979,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
     </font>
   </fonts>
   <fills count="2">
@@ -995,9 +1007,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1359,7 +1372,9 @@
       <c r="J1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="K1" s="1"/>
+      <c r="K1" s="2" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -1392,6 +1407,9 @@
       <c r="J2" t="s">
         <v>230</v>
       </c>
+      <c r="K2">
+        <v>89.7</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -1424,6 +1442,9 @@
       <c r="J3" t="s">
         <v>228</v>
       </c>
+      <c r="K3">
+        <v>100</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -1456,6 +1477,9 @@
       <c r="J4" t="s">
         <v>234</v>
       </c>
+      <c r="K4">
+        <v>100</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -1488,6 +1512,9 @@
       <c r="J5" t="s">
         <v>234</v>
       </c>
+      <c r="K5">
+        <v>92.3</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1520,6 +1547,9 @@
       <c r="J6" t="s">
         <v>237</v>
       </c>
+      <c r="K6">
+        <v>26.9</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1552,6 +1582,9 @@
       <c r="J7" t="s">
         <v>232</v>
       </c>
+      <c r="K7">
+        <v>100</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -1584,6 +1617,9 @@
       <c r="J8" t="s">
         <v>230</v>
       </c>
+      <c r="K8">
+        <v>91.7</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1616,6 +1652,9 @@
       <c r="J9" t="s">
         <v>240</v>
       </c>
+      <c r="K9">
+        <v>69</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -1648,6 +1687,9 @@
       <c r="J10" t="s">
         <v>242</v>
       </c>
+      <c r="K10">
+        <v>100</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -1680,6 +1722,9 @@
       <c r="J11" t="s">
         <v>245</v>
       </c>
+      <c r="K11">
+        <v>95.8</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1712,6 +1757,9 @@
       <c r="J12" t="s">
         <v>124</v>
       </c>
+      <c r="K12">
+        <v>30.4</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -1744,6 +1792,9 @@
       <c r="J13" t="s">
         <v>247</v>
       </c>
+      <c r="K13">
+        <v>100</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1776,6 +1827,9 @@
       <c r="J14" t="s">
         <v>253</v>
       </c>
+      <c r="K14">
+        <v>100</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -1808,6 +1862,9 @@
       <c r="J15" t="s">
         <v>232</v>
       </c>
+      <c r="K15">
+        <v>96</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1840,8 +1897,11 @@
       <c r="J16" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K16">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -1872,8 +1932,11 @@
       <c r="J17" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K17">
+        <v>88.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -1904,8 +1967,11 @@
       <c r="J18" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K18">
+        <v>82.1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>45</v>
       </c>
@@ -1936,8 +2002,11 @@
       <c r="J19" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K19">
+        <v>88.9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>47</v>
       </c>
@@ -1968,8 +2037,11 @@
       <c r="J20" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K20">
+        <v>34.799999999999997</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>49</v>
       </c>
@@ -2000,8 +2072,11 @@
       <c r="J21" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K21">
+        <v>91.7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -2032,8 +2107,11 @@
       <c r="J22" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K22">
+        <v>64.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -2064,8 +2142,11 @@
       <c r="J23" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K23">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -2096,8 +2177,11 @@
       <c r="J24" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K24">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>57</v>
       </c>
@@ -2128,8 +2212,11 @@
       <c r="J25" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K25">
+        <v>89.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>59</v>
       </c>
@@ -2160,8 +2247,11 @@
       <c r="J26" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K26">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>61</v>
       </c>
@@ -2192,8 +2282,11 @@
       <c r="J27" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K27">
+        <v>78.3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>63</v>
       </c>
@@ -2224,8 +2317,11 @@
       <c r="J28" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K28">
+        <v>31.6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>65</v>
       </c>
@@ -2256,8 +2352,11 @@
       <c r="J29" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K29">
+        <v>69.599999999999994</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>67</v>
       </c>
@@ -2288,8 +2387,11 @@
       <c r="J30" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K30">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>69</v>
       </c>
@@ -2320,8 +2422,11 @@
       <c r="J31" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K31">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>71</v>
       </c>
@@ -2352,8 +2457,11 @@
       <c r="J32" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K32">
+        <v>44.4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>73</v>
       </c>
@@ -2384,8 +2492,11 @@
       <c r="J33" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K33">
+        <v>39.1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>75</v>
       </c>
@@ -2416,8 +2527,11 @@
       <c r="J34" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K34">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>77</v>
       </c>
@@ -2448,8 +2562,11 @@
       <c r="J35" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K35">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>79</v>
       </c>
@@ -2480,8 +2597,11 @@
       <c r="J36" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K36">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>81</v>
       </c>
@@ -2512,8 +2632,11 @@
       <c r="J37" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K37">
+        <v>62.1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>83</v>
       </c>
@@ -2544,8 +2667,11 @@
       <c r="J38" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K38">
+        <v>78.3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>85</v>
       </c>
@@ -2576,8 +2702,11 @@
       <c r="J39" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K39">
+        <v>95.7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>87</v>
       </c>
@@ -2608,8 +2737,11 @@
       <c r="J40" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K40">
+        <v>60.9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>89</v>
       </c>
@@ -2640,8 +2772,11 @@
       <c r="J41" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K41">
+        <v>80.8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>91</v>
       </c>
@@ -2672,8 +2807,11 @@
       <c r="J42" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K42">
+        <v>73.099999999999994</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>93</v>
       </c>
@@ -2704,8 +2842,11 @@
       <c r="J43" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K43">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>95</v>
       </c>
@@ -2736,8 +2877,11 @@
       <c r="J44" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K44">
+        <v>23.1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>97</v>
       </c>
@@ -2768,8 +2912,11 @@
       <c r="J45" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K45">
+        <v>79.2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>99</v>
       </c>
@@ -2800,8 +2947,11 @@
       <c r="J46" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K46">
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>101</v>
       </c>
@@ -2832,8 +2982,11 @@
       <c r="J47" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K47">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>103</v>
       </c>
@@ -2864,8 +3017,11 @@
       <c r="J48" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K48">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>105</v>
       </c>
@@ -2896,8 +3052,11 @@
       <c r="J49" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K49">
+        <v>65.2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>107</v>
       </c>
@@ -2928,8 +3087,11 @@
       <c r="J50" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K50">
+        <v>77.3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>109</v>
       </c>
@@ -2960,8 +3122,11 @@
       <c r="J51" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K51">
+        <v>91.7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>111</v>
       </c>
@@ -2992,8 +3157,11 @@
       <c r="J52" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K52">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>113</v>
       </c>
@@ -3024,8 +3192,11 @@
       <c r="J53" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K53">
+        <v>63.2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>115</v>
       </c>
@@ -3055,6 +3226,9 @@
       </c>
       <c r="J54" t="s">
         <v>304</v>
+      </c>
+      <c r="K54">
+        <v>17.399999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>